<commit_message>
Excel: top50→100, orden %NoDispo DESC/Eficacia ASC, formatos %, limpiar ID hotel CR
</commit_message>
<xml_diff>
--- a/checkrates/week-21/Analisis_Checkrates_B2C_7d.xlsx
+++ b/checkrates/week-21/Analisis_Checkrates_B2C_7d.xlsx
@@ -136,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -150,6 +150,8 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -533,7 +535,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:52 · W21 · 18–24 may 2026</t>
+          <t>Generado: 25/05/2026 23:40 · W21 · 18–24 may 2026</t>
         </is>
       </c>
     </row>
@@ -658,7 +660,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:52 · W21 · 18–24 may 2026</t>
+          <t>Generado: 25/05/2026 23:40 · W21 · 18–24 may 2026</t>
         </is>
       </c>
     </row>
@@ -792,7 +794,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:52 · W21 · 18–24 may 2026</t>
+          <t>Generado: 25/05/2026 23:40 · W21 · 18–24 may 2026</t>
         </is>
       </c>
     </row>
@@ -874,19 +876,19 @@
           <t>Cartagena Area</t>
         </is>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="11" t="n">
         <v>342</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="F6" s="11" t="n">
         <v>70</v>
       </c>
-      <c r="G6" s="5" t="n">
+      <c r="G6" s="12" t="n">
         <v>0.2046783625730994</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="H6" s="12" t="n">
         <v>0.002923976608187134</v>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -920,19 +922,19 @@
           <t>Ixtapa / Zihuatanejo</t>
         </is>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="11" t="n">
         <v>639</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" s="11" t="n">
         <v>135</v>
       </c>
-      <c r="G7" s="5" t="n">
+      <c r="G7" s="12" t="n">
         <v>0.2112676056338028</v>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="H7" s="12" t="n">
         <v>0.004694835680751174</v>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -966,19 +968,19 @@
           <t>Las Vegas (and vicinity), NV, US</t>
         </is>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D8" s="11" t="n">
         <v>2827</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F8" s="11" t="n">
         <v>1169</v>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="G8" s="12" t="n">
         <v>0.4135125574814291</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="H8" s="12" t="n">
         <v>0.002476123098691192</v>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -1012,19 +1014,19 @@
           <t>Orlando</t>
         </is>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="D9" s="11" t="n">
         <v>194</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="F9" s="11" t="n">
         <v>117</v>
       </c>
-      <c r="G9" s="5" t="n">
+      <c r="G9" s="12" t="n">
         <v>0.6030927835051546</v>
       </c>
-      <c r="H9" s="5" t="n">
+      <c r="H9" s="12" t="n">
         <v>0.01030927835051546</v>
       </c>
       <c r="I9" s="6" t="inlineStr">
@@ -1060,19 +1062,19 @@
           <t>New York</t>
         </is>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D10" s="11" t="n">
         <v>393</v>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E10" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F10" s="5" t="n">
+      <c r="F10" s="11" t="n">
         <v>253</v>
       </c>
-      <c r="G10" s="5" t="n">
+      <c r="G10" s="12" t="n">
         <v>0.6437659033078881</v>
       </c>
-      <c r="H10" s="5" t="n">
+      <c r="H10" s="12" t="n">
         <v>0.005089058524173028</v>
       </c>
       <c r="I10" s="6" t="inlineStr">
@@ -1108,19 +1110,19 @@
           <t>Acapulco</t>
         </is>
       </c>
-      <c r="D11" s="5" t="n">
+      <c r="D11" s="11" t="n">
         <v>640</v>
       </c>
-      <c r="E11" s="5" t="n">
+      <c r="E11" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="F11" s="11" t="n">
         <v>490</v>
       </c>
-      <c r="G11" s="5" t="n">
+      <c r="G11" s="12" t="n">
         <v>0.765625</v>
       </c>
-      <c r="H11" s="5" t="n">
+      <c r="H11" s="12" t="n">
         <v>0.0171875</v>
       </c>
       <c r="I11" s="6" t="inlineStr">
@@ -1154,19 +1156,19 @@
           <t>Puerto Escondido Area</t>
         </is>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="D12" s="11" t="n">
         <v>153</v>
       </c>
-      <c r="E12" s="5" t="n">
+      <c r="E12" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="F12" s="5" t="n">
+      <c r="F12" s="11" t="n">
         <v>124</v>
       </c>
-      <c r="G12" s="5" t="n">
+      <c r="G12" s="12" t="n">
         <v>0.8104575163398693</v>
       </c>
-      <c r="H12" s="5" t="n">
+      <c r="H12" s="12" t="n">
         <v>0.08496732026143791</v>
       </c>
       <c r="I12" s="6" t="inlineStr">
@@ -1200,19 +1202,19 @@
           <t>Chicago</t>
         </is>
       </c>
-      <c r="D13" s="5" t="n">
+      <c r="D13" s="11" t="n">
         <v>320</v>
       </c>
-      <c r="E13" s="5" t="n">
+      <c r="E13" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F13" s="5" t="n">
+      <c r="F13" s="11" t="n">
         <v>274</v>
       </c>
-      <c r="G13" s="5" t="n">
+      <c r="G13" s="12" t="n">
         <v>0.85625</v>
       </c>
-      <c r="H13" s="5" t="n">
+      <c r="H13" s="12" t="n">
         <v>0.003125</v>
       </c>
       <c r="I13" s="7" t="inlineStr">
@@ -1246,19 +1248,19 @@
           <t>Cancún</t>
         </is>
       </c>
-      <c r="D14" s="5" t="n">
+      <c r="D14" s="11" t="n">
         <v>1718</v>
       </c>
-      <c r="E14" s="5" t="n">
+      <c r="E14" s="11" t="n">
         <v>81</v>
       </c>
-      <c r="F14" s="5" t="n">
+      <c r="F14" s="11" t="n">
         <v>1476</v>
       </c>
-      <c r="G14" s="5" t="n">
+      <c r="G14" s="12" t="n">
         <v>0.8591385331781141</v>
       </c>
-      <c r="H14" s="5" t="n">
+      <c r="H14" s="12" t="n">
         <v>0.04714784633294528</v>
       </c>
       <c r="I14" s="7" t="inlineStr">
@@ -1292,19 +1294,19 @@
           <t>Laughlin Area</t>
         </is>
       </c>
-      <c r="D15" s="5" t="n">
+      <c r="D15" s="11" t="n">
         <v>364</v>
       </c>
-      <c r="E15" s="5" t="n">
+      <c r="E15" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="F15" s="5" t="n">
+      <c r="F15" s="11" t="n">
         <v>319</v>
       </c>
-      <c r="G15" s="5" t="n">
+      <c r="G15" s="12" t="n">
         <v>0.8763736263736264</v>
       </c>
-      <c r="H15" s="5" t="n">
+      <c r="H15" s="12" t="n">
         <v>0.03571428571428571</v>
       </c>
       <c r="I15" s="7" t="inlineStr">
@@ -1360,7 +1362,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:52 · W21 · 18–24 may 2026</t>
+          <t>Generado: 25/05/2026 23:40 · W21 · 18–24 may 2026</t>
         </is>
       </c>
     </row>
@@ -1442,19 +1444,19 @@
           <t>Tokyo</t>
         </is>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="11" t="n">
         <v>7059</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="F6" s="11" t="n">
         <v>6924</v>
       </c>
-      <c r="G6" s="5" t="n">
+      <c r="G6" s="12" t="n">
         <v>0.9808754781130472</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="H6" s="12" t="n">
         <v>0.0001416631250885395</v>
       </c>
       <c r="I6" s="9" t="inlineStr">
@@ -1488,19 +1490,19 @@
           <t>Las Vegas (and vicinity), NV, US</t>
         </is>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="11" t="n">
         <v>2827</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" s="11" t="n">
         <v>1169</v>
       </c>
-      <c r="G7" s="5" t="n">
+      <c r="G7" s="12" t="n">
         <v>0.4135125574814291</v>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="H7" s="12" t="n">
         <v>0.002476123098691192</v>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -1534,19 +1536,19 @@
           <t>Niagara Falls, Canada</t>
         </is>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D8" s="11" t="n">
         <v>2738</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F8" s="11" t="n">
         <v>2723</v>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="G8" s="12" t="n">
         <v>0.9945215485756026</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="H8" s="12" t="n">
         <v>0.001826150474799124</v>
       </c>
       <c r="I8" s="9" t="inlineStr">
@@ -1578,19 +1580,19 @@
           <t>Paris</t>
         </is>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="D9" s="11" t="n">
         <v>1321</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="F9" s="11" t="n">
         <v>1244</v>
       </c>
-      <c r="G9" s="5" t="n">
+      <c r="G9" s="12" t="n">
         <v>0.9417108251324754</v>
       </c>
-      <c r="H9" s="5" t="n">
+      <c r="H9" s="12" t="n">
         <v>0.001514004542013626</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
@@ -1624,19 +1626,19 @@
           <t>Las Vegas (and vicinity), NV, US</t>
         </is>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D10" s="11" t="n">
         <v>1163</v>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E10" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F10" s="5" t="n">
+      <c r="F10" s="11" t="n">
         <v>1151</v>
       </c>
-      <c r="G10" s="5" t="n">
+      <c r="G10" s="12" t="n">
         <v>0.9896818572656921</v>
       </c>
-      <c r="H10" s="5" t="n">
+      <c r="H10" s="12" t="n">
         <v>0.002579535683576956</v>
       </c>
       <c r="I10" s="9" t="inlineStr">
@@ -1668,19 +1670,19 @@
           <t>Las Vegas (and vicinity), NV, US</t>
         </is>
       </c>
-      <c r="D11" s="5" t="n">
+      <c r="D11" s="11" t="n">
         <v>1124</v>
       </c>
-      <c r="E11" s="5" t="n">
+      <c r="E11" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="F11" s="11" t="n">
         <v>1123</v>
       </c>
-      <c r="G11" s="5" t="n">
+      <c r="G11" s="12" t="n">
         <v>0.9991103202846975</v>
       </c>
-      <c r="H11" s="5" t="n">
+      <c r="H11" s="12" t="n">
         <v>0.001779359430604982</v>
       </c>
       <c r="I11" s="9" t="inlineStr">
@@ -1712,19 +1714,19 @@
           <t>Las Vegas (and vicinity), NV, US</t>
         </is>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="D12" s="11" t="n">
         <v>1093</v>
       </c>
-      <c r="E12" s="5" t="n">
+      <c r="E12" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="F12" s="5" t="n">
+      <c r="F12" s="11" t="n">
         <v>1074</v>
       </c>
-      <c r="G12" s="5" t="n">
+      <c r="G12" s="12" t="n">
         <v>0.9826166514181153</v>
       </c>
-      <c r="H12" s="5" t="n">
+      <c r="H12" s="12" t="n">
         <v>0.006404391582799634</v>
       </c>
       <c r="I12" s="9" t="inlineStr">
@@ -1756,19 +1758,19 @@
           <t>Honolulu Area</t>
         </is>
       </c>
-      <c r="D13" s="5" t="n">
+      <c r="D13" s="11" t="n">
         <v>1004</v>
       </c>
-      <c r="E13" s="5" t="n">
+      <c r="E13" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F13" s="5" t="n">
+      <c r="F13" s="11" t="n">
         <v>997</v>
       </c>
-      <c r="G13" s="5" t="n">
+      <c r="G13" s="12" t="n">
         <v>0.9930278884462151</v>
       </c>
-      <c r="H13" s="5" t="n">
+      <c r="H13" s="12" t="n">
         <v>0.00199203187250996</v>
       </c>
       <c r="I13" s="9" t="inlineStr">
@@ -1800,19 +1802,19 @@
           <t>Las Vegas (and vicinity), NV, US</t>
         </is>
       </c>
-      <c r="D14" s="5" t="n">
+      <c r="D14" s="11" t="n">
         <v>764</v>
       </c>
-      <c r="E14" s="5" t="n">
+      <c r="E14" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="F14" s="5" t="n">
+      <c r="F14" s="11" t="n">
         <v>751</v>
       </c>
-      <c r="G14" s="5" t="n">
+      <c r="G14" s="12" t="n">
         <v>0.9829842931937173</v>
       </c>
-      <c r="H14" s="5" t="n">
+      <c r="H14" s="12" t="n">
         <v>0.01047120418848168</v>
       </c>
       <c r="I14" s="9" t="inlineStr">
@@ -1844,19 +1846,19 @@
           <t>Las Vegas (and vicinity), NV, US</t>
         </is>
       </c>
-      <c r="D15" s="5" t="n">
+      <c r="D15" s="11" t="n">
         <v>719</v>
       </c>
-      <c r="E15" s="5" t="n">
+      <c r="E15" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F15" s="5" t="n">
+      <c r="F15" s="11" t="n">
         <v>714</v>
       </c>
-      <c r="G15" s="5" t="n">
+      <c r="G15" s="12" t="n">
         <v>0.9930458970792768</v>
       </c>
-      <c r="H15" s="5" t="n">
+      <c r="H15" s="12" t="n">
         <v>0.001390820584144645</v>
       </c>
       <c r="I15" s="9" t="inlineStr">
@@ -1910,7 +1912,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:52 · W21 · 18–24 may 2026</t>
+          <t>Generado: 25/05/2026 23:40 · W21 · 18–24 may 2026</t>
         </is>
       </c>
     </row>
@@ -1992,19 +1994,19 @@
           <t>Paris</t>
         </is>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="11" t="n">
         <v>3012</v>
       </c>
-      <c r="E6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="5" t="n">
+      <c r="E6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="11" t="n">
         <v>2949</v>
       </c>
-      <c r="G6" s="5" t="n">
+      <c r="G6" s="12" t="n">
         <v>0.9790836653386454</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="H6" s="12" t="n">
         <v>0</v>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -2038,19 +2040,19 @@
           <t>Paris</t>
         </is>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="11" t="n">
         <v>2379</v>
       </c>
-      <c r="E7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="5" t="n">
+      <c r="E7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="11" t="n">
         <v>2313</v>
       </c>
-      <c r="G7" s="5" t="n">
+      <c r="G7" s="12" t="n">
         <v>0.9722572509457755</v>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="H7" s="12" t="n">
         <v>0</v>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -2084,19 +2086,19 @@
           <t>Las Vegas (and vicinity), NV, US</t>
         </is>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D8" s="11" t="n">
         <v>2328</v>
       </c>
-      <c r="E8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="5" t="n">
+      <c r="E8" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="11" t="n">
         <v>296</v>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="G8" s="12" t="n">
         <v>0.127147766323024</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="H8" s="12" t="n">
         <v>0</v>
       </c>
       <c r="I8" s="5" t="inlineStr">
@@ -2128,19 +2130,19 @@
           <t>New York</t>
         </is>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="D9" s="11" t="n">
         <v>1938</v>
       </c>
-      <c r="E9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="5" t="n">
+      <c r="E9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="11" t="n">
         <v>1871</v>
       </c>
-      <c r="G9" s="5" t="n">
+      <c r="G9" s="12" t="n">
         <v>0.9654282765737874</v>
       </c>
-      <c r="H9" s="5" t="n">
+      <c r="H9" s="12" t="n">
         <v>0</v>
       </c>
       <c r="I9" s="5" t="inlineStr">
@@ -2174,19 +2176,19 @@
           <t>Chicago</t>
         </is>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D10" s="11" t="n">
         <v>1829</v>
       </c>
-      <c r="E10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="5" t="n">
+      <c r="E10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="11" t="n">
         <v>1786</v>
       </c>
-      <c r="G10" s="5" t="n">
+      <c r="G10" s="12" t="n">
         <v>0.9764898851831602</v>
       </c>
-      <c r="H10" s="5" t="n">
+      <c r="H10" s="12" t="n">
         <v>0</v>
       </c>
       <c r="I10" s="5" t="inlineStr">
@@ -2218,19 +2220,19 @@
           <t>Las Vegas (and vicinity), NV, US</t>
         </is>
       </c>
-      <c r="D11" s="5" t="n">
+      <c r="D11" s="11" t="n">
         <v>1682</v>
       </c>
-      <c r="E11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="5" t="n">
+      <c r="E11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="11" t="n">
         <v>277</v>
       </c>
-      <c r="G11" s="5" t="n">
+      <c r="G11" s="12" t="n">
         <v>0.1646848989298454</v>
       </c>
-      <c r="H11" s="5" t="n">
+      <c r="H11" s="12" t="n">
         <v>0</v>
       </c>
       <c r="I11" s="5" t="inlineStr">
@@ -2262,19 +2264,19 @@
           <t>Los Angeles (and vicinity), CA, US</t>
         </is>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="D12" s="11" t="n">
         <v>1462</v>
       </c>
-      <c r="E12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="5" t="n">
+      <c r="E12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="11" t="n">
         <v>1446</v>
       </c>
-      <c r="G12" s="5" t="n">
+      <c r="G12" s="12" t="n">
         <v>0.9890560875512996</v>
       </c>
-      <c r="H12" s="5" t="n">
+      <c r="H12" s="12" t="n">
         <v>0</v>
       </c>
       <c r="I12" s="5" t="inlineStr">
@@ -2308,19 +2310,19 @@
           <t>El Cairo Area</t>
         </is>
       </c>
-      <c r="D13" s="5" t="n">
+      <c r="D13" s="11" t="n">
         <v>1185</v>
       </c>
-      <c r="E13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="5" t="n">
+      <c r="E13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="11" t="n">
         <v>1170</v>
       </c>
-      <c r="G13" s="5" t="n">
+      <c r="G13" s="12" t="n">
         <v>0.9873417721518988</v>
       </c>
-      <c r="H13" s="5" t="n">
+      <c r="H13" s="12" t="n">
         <v>0</v>
       </c>
       <c r="I13" s="5" t="inlineStr">
@@ -2352,19 +2354,19 @@
           <t>Paris</t>
         </is>
       </c>
-      <c r="D14" s="5" t="n">
+      <c r="D14" s="11" t="n">
         <v>1171</v>
       </c>
-      <c r="E14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="5" t="n">
+      <c r="E14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="11" t="n">
         <v>1154</v>
       </c>
-      <c r="G14" s="5" t="n">
+      <c r="G14" s="12" t="n">
         <v>0.9854824935952178</v>
       </c>
-      <c r="H14" s="5" t="n">
+      <c r="H14" s="12" t="n">
         <v>0</v>
       </c>
       <c r="I14" s="5" t="inlineStr">
@@ -2398,19 +2400,19 @@
           <t>Budapest Area</t>
         </is>
       </c>
-      <c r="D15" s="5" t="n">
+      <c r="D15" s="11" t="n">
         <v>1017</v>
       </c>
-      <c r="E15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="5" t="n">
+      <c r="E15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="11" t="n">
         <v>996</v>
       </c>
-      <c r="G15" s="5" t="n">
+      <c r="G15" s="12" t="n">
         <v>0.9793510324483776</v>
       </c>
-      <c r="H15" s="5" t="n">
+      <c r="H15" s="12" t="n">
         <v>0</v>
       </c>
       <c r="I15" s="5" t="inlineStr">
@@ -2464,7 +2466,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:52 · W21 · 18–24 may 2026</t>
+          <t>Generado: 25/05/2026 23:40 · W21 · 18–24 may 2026</t>
         </is>
       </c>
     </row>
@@ -2546,19 +2548,19 @@
           <t>Tokyo</t>
         </is>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="11" t="n">
         <v>7059</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="F6" s="11" t="n">
         <v>6924</v>
       </c>
-      <c r="G6" s="5" t="n">
+      <c r="G6" s="12" t="n">
         <v>0.9808754781130472</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="H6" s="12" t="n">
         <v>0.0001416631250885395</v>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -2592,19 +2594,19 @@
           <t>Las Vegas (and vicinity), NV, US</t>
         </is>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="11" t="n">
         <v>719</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" s="11" t="n">
         <v>714</v>
       </c>
-      <c r="G7" s="5" t="n">
+      <c r="G7" s="12" t="n">
         <v>0.9930458970792768</v>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="H7" s="12" t="n">
         <v>0.001390820584144645</v>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -2636,19 +2638,19 @@
           <t>Paris</t>
         </is>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D8" s="11" t="n">
         <v>1321</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F8" s="11" t="n">
         <v>1244</v>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="G8" s="12" t="n">
         <v>0.9417108251324754</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="H8" s="12" t="n">
         <v>0.001514004542013626</v>
       </c>
       <c r="I8" s="5" t="inlineStr">
@@ -2682,19 +2684,19 @@
           <t>Las Vegas (and vicinity), NV, US</t>
         </is>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="D9" s="11" t="n">
         <v>1124</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="F9" s="11" t="n">
         <v>1123</v>
       </c>
-      <c r="G9" s="5" t="n">
+      <c r="G9" s="12" t="n">
         <v>0.9991103202846975</v>
       </c>
-      <c r="H9" s="5" t="n">
+      <c r="H9" s="12" t="n">
         <v>0.001779359430604982</v>
       </c>
       <c r="I9" s="5" t="inlineStr">
@@ -2726,19 +2728,19 @@
           <t>Niagara Falls, Canada</t>
         </is>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D10" s="11" t="n">
         <v>2738</v>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E10" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="F10" s="5" t="n">
+      <c r="F10" s="11" t="n">
         <v>2723</v>
       </c>
-      <c r="G10" s="5" t="n">
+      <c r="G10" s="12" t="n">
         <v>0.9945215485756026</v>
       </c>
-      <c r="H10" s="5" t="n">
+      <c r="H10" s="12" t="n">
         <v>0.001826150474799124</v>
       </c>
       <c r="I10" s="5" t="inlineStr">
@@ -2770,19 +2772,19 @@
           <t>Las Vegas (and vicinity), NV, US</t>
         </is>
       </c>
-      <c r="D11" s="5" t="n">
+      <c r="D11" s="11" t="n">
         <v>541</v>
       </c>
-      <c r="E11" s="5" t="n">
+      <c r="E11" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="F11" s="11" t="n">
         <v>534</v>
       </c>
-      <c r="G11" s="5" t="n">
+      <c r="G11" s="12" t="n">
         <v>0.9870609981515711</v>
       </c>
-      <c r="H11" s="5" t="n">
+      <c r="H11" s="12" t="n">
         <v>0.001848428835489834</v>
       </c>
       <c r="I11" s="5" t="inlineStr">
@@ -2814,19 +2816,19 @@
           <t>Honolulu Area</t>
         </is>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="D12" s="11" t="n">
         <v>1004</v>
       </c>
-      <c r="E12" s="5" t="n">
+      <c r="E12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F12" s="5" t="n">
+      <c r="F12" s="11" t="n">
         <v>997</v>
       </c>
-      <c r="G12" s="5" t="n">
+      <c r="G12" s="12" t="n">
         <v>0.9930278884462151</v>
       </c>
-      <c r="H12" s="5" t="n">
+      <c r="H12" s="12" t="n">
         <v>0.00199203187250996</v>
       </c>
       <c r="I12" s="5" t="inlineStr">
@@ -2858,19 +2860,19 @@
           <t>Las Vegas (and vicinity), NV, US</t>
         </is>
       </c>
-      <c r="D13" s="5" t="n">
+      <c r="D13" s="11" t="n">
         <v>487</v>
       </c>
-      <c r="E13" s="5" t="n">
+      <c r="E13" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F13" s="5" t="n">
+      <c r="F13" s="11" t="n">
         <v>485</v>
       </c>
-      <c r="G13" s="5" t="n">
+      <c r="G13" s="12" t="n">
         <v>0.9958932238193019</v>
       </c>
-      <c r="H13" s="5" t="n">
+      <c r="H13" s="12" t="n">
         <v>0.002053388090349076</v>
       </c>
       <c r="I13" s="5" t="inlineStr">
@@ -2902,19 +2904,19 @@
           <t>New York</t>
         </is>
       </c>
-      <c r="D14" s="5" t="n">
+      <c r="D14" s="11" t="n">
         <v>423</v>
       </c>
-      <c r="E14" s="5" t="n">
+      <c r="E14" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F14" s="5" t="n">
+      <c r="F14" s="11" t="n">
         <v>423</v>
       </c>
-      <c r="G14" s="5" t="n">
+      <c r="G14" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H14" s="5" t="n">
+      <c r="H14" s="12" t="n">
         <v>0.002364066193853428</v>
       </c>
       <c r="I14" s="5" t="inlineStr">
@@ -2946,19 +2948,19 @@
           <t>Las Vegas (and vicinity), NV, US</t>
         </is>
       </c>
-      <c r="D15" s="5" t="n">
+      <c r="D15" s="11" t="n">
         <v>2827</v>
       </c>
-      <c r="E15" s="5" t="n">
+      <c r="E15" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="F15" s="5" t="n">
+      <c r="F15" s="11" t="n">
         <v>1169</v>
       </c>
-      <c r="G15" s="5" t="n">
+      <c r="G15" s="12" t="n">
         <v>0.4135125574814291</v>
       </c>
-      <c r="H15" s="5" t="n">
+      <c r="H15" s="12" t="n">
         <v>0.002476123098691192</v>
       </c>
       <c r="I15" s="5" t="inlineStr">
@@ -3010,7 +3012,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:52 · W21 · 18–24 may 2026</t>
+          <t>Generado: 25/05/2026 23:40 · W21 · 18–24 may 2026</t>
         </is>
       </c>
     </row>
@@ -3062,19 +3064,19 @@
           <t>Hyatt</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="11" t="n">
         <v>29534</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="11" t="n">
         <v>14</v>
       </c>
       <c r="D6" s="5" t="n">
         <v>28265</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="12" t="n">
         <v>0.9570325726281573</v>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="F6" s="12" t="n">
         <v>0.0004740299316042527</v>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -3094,19 +3096,19 @@
           <t>Hilton</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B7" s="11" t="n">
         <v>18361</v>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="11" t="n">
         <v>7</v>
       </c>
       <c r="D7" s="5" t="n">
         <v>18181</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="12" t="n">
         <v>0.9901966123849464</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" s="12" t="n">
         <v>0.0003812428516965307</v>
       </c>
       <c r="G7" s="5" t="inlineStr">
@@ -3126,19 +3128,19 @@
           <t>IHG</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="11" t="n">
         <v>14225</v>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="11" t="n">
         <v>1</v>
       </c>
       <c r="D8" s="5" t="n">
         <v>14027</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="12" t="n">
         <v>0.9860808435852373</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F8" s="12" t="n">
         <v>7.0298769771529e-05</v>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -3158,19 +3160,19 @@
           <t>AA-Independent</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="11" t="n">
         <v>13312</v>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="11" t="n">
         <v>229</v>
       </c>
       <c r="D9" s="5" t="n">
         <v>7884</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="12" t="n">
         <v>0.5922475961538461</v>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="F9" s="12" t="n">
         <v>0.01720252403846154</v>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -3190,19 +3192,19 @@
           <t>Accor</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" s="11" t="n">
         <v>10033</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="11" t="n">
         <v>18</v>
       </c>
       <c r="D10" s="5" t="n">
         <v>9445</v>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E10" s="12" t="n">
         <v>0.9413934017741453</v>
       </c>
-      <c r="F10" s="5" t="n">
+      <c r="F10" s="12" t="n">
         <v>0.001794079537526164</v>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -3222,19 +3224,19 @@
           <t>Caesars Entertainment</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n">
+      <c r="B11" s="11" t="n">
         <v>7670</v>
       </c>
-      <c r="C11" s="5" t="n">
+      <c r="C11" s="11" t="n">
         <v>35</v>
       </c>
       <c r="D11" s="5" t="n">
         <v>5942</v>
       </c>
-      <c r="E11" s="5" t="n">
+      <c r="E11" s="12" t="n">
         <v>0.7747066492829204</v>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="F11" s="12" t="n">
         <v>0.004563233376792698</v>
       </c>
       <c r="G11" s="5" t="inlineStr">
@@ -3254,19 +3256,19 @@
           <t>Hyatt Inclusive Collection</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n">
+      <c r="B12" s="11" t="n">
         <v>4518</v>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C12" s="11" t="n">
         <v>4</v>
       </c>
       <c r="D12" s="5" t="n">
         <v>4396</v>
       </c>
-      <c r="E12" s="5" t="n">
+      <c r="E12" s="12" t="n">
         <v>0.9729969012837538</v>
       </c>
-      <c r="F12" s="5" t="n">
+      <c r="F12" s="12" t="n">
         <v>0.0008853474988933156</v>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -3286,19 +3288,19 @@
           <t>MGM Resorts</t>
         </is>
       </c>
-      <c r="B13" s="5" t="n">
+      <c r="B13" s="11" t="n">
         <v>3272</v>
       </c>
-      <c r="C13" s="5" t="n">
+      <c r="C13" s="11" t="n">
         <v>17</v>
       </c>
       <c r="D13" s="5" t="n">
         <v>3208</v>
       </c>
-      <c r="E13" s="5" t="n">
+      <c r="E13" s="12" t="n">
         <v>0.980440097799511</v>
       </c>
-      <c r="F13" s="5" t="n">
+      <c r="F13" s="12" t="n">
         <v>0.00519559902200489</v>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -3318,19 +3320,19 @@
           <t>Wyndham</t>
         </is>
       </c>
-      <c r="B14" s="5" t="n">
+      <c r="B14" s="11" t="n">
         <v>1427</v>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="C14" s="11" t="n">
         <v>5</v>
       </c>
       <c r="D14" s="5" t="n">
         <v>1372</v>
       </c>
-      <c r="E14" s="5" t="n">
+      <c r="E14" s="12" t="n">
         <v>0.9614576033637001</v>
       </c>
-      <c r="F14" s="5" t="n">
+      <c r="F14" s="12" t="n">
         <v>0.00350385423966363</v>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -3350,19 +3352,19 @@
           <t>Disney</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n">
+      <c r="B15" s="11" t="n">
         <v>1027</v>
       </c>
-      <c r="C15" s="5" t="n">
+      <c r="C15" s="11" t="n">
         <v>6</v>
       </c>
       <c r="D15" s="5" t="n">
         <v>1021</v>
       </c>
-      <c r="E15" s="5" t="n">
+      <c r="E15" s="12" t="n">
         <v>0.994157740993184</v>
       </c>
-      <c r="F15" s="5" t="n">
+      <c r="F15" s="12" t="n">
         <v>0.005842259006815969</v>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -3382,19 +3384,19 @@
           <t>Palace</t>
         </is>
       </c>
-      <c r="B16" s="5" t="n">
+      <c r="B16" s="11" t="n">
         <v>707</v>
       </c>
-      <c r="C16" s="5" t="n">
+      <c r="C16" s="11" t="n">
         <v>2</v>
       </c>
       <c r="D16" s="5" t="n">
         <v>705</v>
       </c>
-      <c r="E16" s="5" t="n">
+      <c r="E16" s="12" t="n">
         <v>0.9971711456859972</v>
       </c>
-      <c r="F16" s="5" t="n">
+      <c r="F16" s="12" t="n">
         <v>0.002828854314002829</v>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -3414,19 +3416,19 @@
           <t>Universal</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n">
+      <c r="B17" s="11" t="n">
         <v>694</v>
       </c>
-      <c r="C17" s="5" t="n">
+      <c r="C17" s="11" t="n">
         <v>8</v>
       </c>
       <c r="D17" s="5" t="n">
         <v>685</v>
       </c>
-      <c r="E17" s="5" t="n">
+      <c r="E17" s="12" t="n">
         <v>0.9870317002881844</v>
       </c>
-      <c r="F17" s="5" t="n">
+      <c r="F17" s="12" t="n">
         <v>0.01152737752161383</v>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -3446,19 +3448,19 @@
           <t>Wynn Las Vegas</t>
         </is>
       </c>
-      <c r="B18" s="5" t="n">
+      <c r="B18" s="11" t="n">
         <v>547</v>
       </c>
-      <c r="C18" s="5" t="n">
+      <c r="C18" s="11" t="n">
         <v>4</v>
       </c>
       <c r="D18" s="5" t="n">
         <v>547</v>
       </c>
-      <c r="E18" s="5" t="n">
+      <c r="E18" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F18" s="5" t="n">
+      <c r="F18" s="12" t="n">
         <v>0.007312614259597806</v>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -3478,19 +3480,19 @@
           <t>Presidente Intercontinental</t>
         </is>
       </c>
-      <c r="B19" s="5" t="n">
+      <c r="B19" s="11" t="n">
         <v>476</v>
       </c>
-      <c r="C19" s="5" t="n">
+      <c r="C19" s="11" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="5" t="n">
         <v>474</v>
       </c>
-      <c r="E19" s="5" t="n">
+      <c r="E19" s="12" t="n">
         <v>0.9957983193277311</v>
       </c>
-      <c r="F19" s="5" t="n">
+      <c r="F19" s="12" t="n">
         <v>0.002100840336134454</v>
       </c>
       <c r="G19" s="5" t="inlineStr">
@@ -3510,19 +3512,19 @@
           <t>Best Western</t>
         </is>
       </c>
-      <c r="B20" s="5" t="n">
+      <c r="B20" s="11" t="n">
         <v>452</v>
       </c>
-      <c r="C20" s="5" t="n">
+      <c r="C20" s="11" t="n">
         <v>2</v>
       </c>
       <c r="D20" s="5" t="n">
         <v>375</v>
       </c>
-      <c r="E20" s="5" t="n">
+      <c r="E20" s="12" t="n">
         <v>0.8296460176991151</v>
       </c>
-      <c r="F20" s="5" t="n">
+      <c r="F20" s="12" t="n">
         <v>0.004424778761061947</v>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -3542,19 +3544,19 @@
           <t>CHOICE</t>
         </is>
       </c>
-      <c r="B21" s="5" t="n">
+      <c r="B21" s="11" t="n">
         <v>445</v>
       </c>
-      <c r="C21" s="5" t="n">
+      <c r="C21" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D21" s="5" t="n">
         <v>444</v>
       </c>
-      <c r="E21" s="5" t="n">
+      <c r="E21" s="12" t="n">
         <v>0.9977528089887641</v>
       </c>
-      <c r="F21" s="5" t="n">
+      <c r="F21" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G21" s="5" t="inlineStr">
@@ -3574,19 +3576,19 @@
           <t>Camino Real</t>
         </is>
       </c>
-      <c r="B22" s="5" t="n">
+      <c r="B22" s="11" t="n">
         <v>391</v>
       </c>
-      <c r="C22" s="5" t="n">
+      <c r="C22" s="11" t="n">
         <v>39</v>
       </c>
       <c r="D22" s="5" t="n">
         <v>391</v>
       </c>
-      <c r="E22" s="5" t="n">
+      <c r="E22" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F22" s="5" t="n">
+      <c r="F22" s="12" t="n">
         <v>0.09974424552429667</v>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -3606,19 +3608,19 @@
           <t>Sandos</t>
         </is>
       </c>
-      <c r="B23" s="5" t="n">
+      <c r="B23" s="11" t="n">
         <v>278</v>
       </c>
-      <c r="C23" s="5" t="n">
+      <c r="C23" s="11" t="n">
         <v>3</v>
       </c>
       <c r="D23" s="5" t="n">
         <v>278</v>
       </c>
-      <c r="E23" s="5" t="n">
+      <c r="E23" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F23" s="5" t="n">
+      <c r="F23" s="12" t="n">
         <v>0.01079136690647482</v>
       </c>
       <c r="G23" s="5" t="inlineStr">
@@ -3638,19 +3640,19 @@
           <t>Decameron</t>
         </is>
       </c>
-      <c r="B24" s="5" t="n">
+      <c r="B24" s="11" t="n">
         <v>268</v>
       </c>
-      <c r="C24" s="5" t="n">
+      <c r="C24" s="11" t="n">
         <v>7</v>
       </c>
       <c r="D24" s="5" t="n">
         <v>241</v>
       </c>
-      <c r="E24" s="5" t="n">
+      <c r="E24" s="12" t="n">
         <v>0.8992537313432836</v>
       </c>
-      <c r="F24" s="5" t="n">
+      <c r="F24" s="12" t="n">
         <v>0.02611940298507463</v>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -3670,19 +3672,19 @@
           <t>Oasis</t>
         </is>
       </c>
-      <c r="B25" s="5" t="n">
+      <c r="B25" s="11" t="n">
         <v>233</v>
       </c>
-      <c r="C25" s="5" t="n">
+      <c r="C25" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D25" s="5" t="n">
         <v>233</v>
       </c>
-      <c r="E25" s="5" t="n">
+      <c r="E25" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F25" s="5" t="n">
+      <c r="F25" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -3702,19 +3704,19 @@
           <t>PAM Hotels</t>
         </is>
       </c>
-      <c r="B26" s="5" t="n">
+      <c r="B26" s="11" t="n">
         <v>216</v>
       </c>
-      <c r="C26" s="5" t="n">
+      <c r="C26" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="5" t="n">
         <v>214</v>
       </c>
-      <c r="E26" s="5" t="n">
+      <c r="E26" s="12" t="n">
         <v>0.9907407407407407</v>
       </c>
-      <c r="F26" s="5" t="n">
+      <c r="F26" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -3734,19 +3736,19 @@
           <t>Hoteles Xcaret</t>
         </is>
       </c>
-      <c r="B27" s="5" t="n">
+      <c r="B27" s="11" t="n">
         <v>193</v>
       </c>
-      <c r="C27" s="5" t="n">
+      <c r="C27" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="5" t="n">
         <v>193</v>
       </c>
-      <c r="E27" s="5" t="n">
+      <c r="E27" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F27" s="5" t="n">
+      <c r="F27" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G27" s="5" t="inlineStr">
@@ -3766,19 +3768,19 @@
           <t>Karisma</t>
         </is>
       </c>
-      <c r="B28" s="5" t="n">
+      <c r="B28" s="11" t="n">
         <v>177</v>
       </c>
-      <c r="C28" s="5" t="n">
+      <c r="C28" s="11" t="n">
         <v>1</v>
       </c>
       <c r="D28" s="5" t="n">
         <v>176</v>
       </c>
-      <c r="E28" s="5" t="n">
+      <c r="E28" s="12" t="n">
         <v>0.9943502824858758</v>
       </c>
-      <c r="F28" s="5" t="n">
+      <c r="F28" s="12" t="n">
         <v>0.005649717514124294</v>
       </c>
       <c r="G28" s="5" t="inlineStr">
@@ -3798,19 +3800,19 @@
           <t>EM Hotels</t>
         </is>
       </c>
-      <c r="B29" s="5" t="n">
+      <c r="B29" s="11" t="n">
         <v>160</v>
       </c>
-      <c r="C29" s="5" t="n">
+      <c r="C29" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D29" s="5" t="n">
         <v>160</v>
       </c>
-      <c r="E29" s="5" t="n">
+      <c r="E29" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F29" s="5" t="n">
+      <c r="F29" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G29" s="5" t="inlineStr">
@@ -3830,19 +3832,19 @@
           <t>Krystal</t>
         </is>
       </c>
-      <c r="B30" s="5" t="n">
+      <c r="B30" s="11" t="n">
         <v>157</v>
       </c>
-      <c r="C30" s="5" t="n">
+      <c r="C30" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E30" s="5" t="n">
+      <c r="E30" s="12" t="n">
         <v>0.01273885350318471</v>
       </c>
-      <c r="F30" s="5" t="n">
+      <c r="F30" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G30" s="5" t="inlineStr">
@@ -3890,7 +3892,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:52 · W21 · 18–24 may 2026</t>
+          <t>Generado: 25/05/2026 23:40 · W21 · 18–24 may 2026</t>
         </is>
       </c>
     </row>
@@ -3942,19 +3944,19 @@
           <t>Las Vegas (and vicinity), NV, US</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="11" t="n">
         <v>17675</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="11" t="n">
         <v>48</v>
       </c>
       <c r="D6" s="5" t="n">
         <v>12322</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="12" t="n">
         <v>0.6971428571428572</v>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="F6" s="12" t="n">
         <v>0.002715700141442716</v>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -3974,19 +3976,19 @@
           <t>New York</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B7" s="11" t="n">
         <v>8675</v>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="11" t="n">
         <v>3</v>
       </c>
       <c r="D7" s="5" t="n">
         <v>8349</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="12" t="n">
         <v>0.9624207492795389</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" s="12" t="n">
         <v>0.000345821325648415</v>
       </c>
       <c r="G7" s="5" t="inlineStr">
@@ -4006,19 +4008,19 @@
           <t>Paris</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="11" t="n">
         <v>8248</v>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="11" t="n">
         <v>2</v>
       </c>
       <c r="D8" s="5" t="n">
         <v>8021</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="12" t="n">
         <v>0.972478176527643</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F8" s="12" t="n">
         <v>0.0002424830261881668</v>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -4038,19 +4040,19 @@
           <t>Tokyo</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="11" t="n">
         <v>7714</v>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="11" t="n">
         <v>2</v>
       </c>
       <c r="D9" s="5" t="n">
         <v>7571</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="12" t="n">
         <v>0.9814622763806067</v>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="F9" s="12" t="n">
         <v>0.0002592688618096966</v>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -4070,19 +4072,19 @@
           <t>Cancún</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" s="11" t="n">
         <v>6356</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="11" t="n">
         <v>94</v>
       </c>
       <c r="D10" s="5" t="n">
         <v>5605</v>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E10" s="12" t="n">
         <v>0.881843926998112</v>
       </c>
-      <c r="F10" s="5" t="n">
+      <c r="F10" s="12" t="n">
         <v>0.01478917558212712</v>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -4102,19 +4104,19 @@
           <t>Chicago</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n">
+      <c r="B11" s="11" t="n">
         <v>4603</v>
       </c>
-      <c r="C11" s="5" t="n">
+      <c r="C11" s="11" t="n">
         <v>1</v>
       </c>
       <c r="D11" s="5" t="n">
         <v>4294</v>
       </c>
-      <c r="E11" s="5" t="n">
+      <c r="E11" s="12" t="n">
         <v>0.9328698674777319</v>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="F11" s="12" t="n">
         <v>0.0002172496198131653</v>
       </c>
       <c r="G11" s="5" t="inlineStr">
@@ -4134,19 +4136,19 @@
           <t>Orlando</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n">
+      <c r="B12" s="11" t="n">
         <v>4058</v>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C12" s="11" t="n">
         <v>17</v>
       </c>
       <c r="D12" s="5" t="n">
         <v>3892</v>
       </c>
-      <c r="E12" s="5" t="n">
+      <c r="E12" s="12" t="n">
         <v>0.9590931493346476</v>
       </c>
-      <c r="F12" s="5" t="n">
+      <c r="F12" s="12" t="n">
         <v>0.004189255791030064</v>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -4166,19 +4168,19 @@
           <t>Niagara Falls, Canada</t>
         </is>
       </c>
-      <c r="B13" s="5" t="n">
+      <c r="B13" s="11" t="n">
         <v>2905</v>
       </c>
-      <c r="C13" s="5" t="n">
+      <c r="C13" s="11" t="n">
         <v>5</v>
       </c>
       <c r="D13" s="5" t="n">
         <v>2883</v>
       </c>
-      <c r="E13" s="5" t="n">
+      <c r="E13" s="12" t="n">
         <v>0.9924268502581756</v>
       </c>
-      <c r="F13" s="5" t="n">
+      <c r="F13" s="12" t="n">
         <v>0.001721170395869191</v>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -4198,19 +4200,19 @@
           <t>Boston</t>
         </is>
       </c>
-      <c r="B14" s="5" t="n">
+      <c r="B14" s="11" t="n">
         <v>2409</v>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="C14" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="5" t="n">
         <v>2355</v>
       </c>
-      <c r="E14" s="5" t="n">
+      <c r="E14" s="12" t="n">
         <v>0.9775840597758406</v>
       </c>
-      <c r="F14" s="5" t="n">
+      <c r="F14" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -4230,19 +4232,19 @@
           <t>Toronto Area</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n">
+      <c r="B15" s="11" t="n">
         <v>2173</v>
       </c>
-      <c r="C15" s="5" t="n">
+      <c r="C15" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D15" s="5" t="n">
         <v>2091</v>
       </c>
-      <c r="E15" s="5" t="n">
+      <c r="E15" s="12" t="n">
         <v>0.9622641509433962</v>
       </c>
-      <c r="F15" s="5" t="n">
+      <c r="F15" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -4262,19 +4264,19 @@
           <t>Honolulu Area</t>
         </is>
       </c>
-      <c r="B16" s="5" t="n">
+      <c r="B16" s="11" t="n">
         <v>2132</v>
       </c>
-      <c r="C16" s="5" t="n">
+      <c r="C16" s="11" t="n">
         <v>2</v>
       </c>
       <c r="D16" s="5" t="n">
         <v>2105</v>
       </c>
-      <c r="E16" s="5" t="n">
+      <c r="E16" s="12" t="n">
         <v>0.9873358348968105</v>
       </c>
-      <c r="F16" s="5" t="n">
+      <c r="F16" s="12" t="n">
         <v>0.0009380863039399625</v>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -4294,19 +4296,19 @@
           <t>Riviera Maya</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n">
+      <c r="B17" s="11" t="n">
         <v>1937</v>
       </c>
-      <c r="C17" s="5" t="n">
+      <c r="C17" s="11" t="n">
         <v>5</v>
       </c>
       <c r="D17" s="5" t="n">
         <v>1847</v>
       </c>
-      <c r="E17" s="5" t="n">
+      <c r="E17" s="12" t="n">
         <v>0.9535363964894166</v>
       </c>
-      <c r="F17" s="5" t="n">
+      <c r="F17" s="12" t="n">
         <v>0.002581311306143521</v>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -4326,19 +4328,19 @@
           <t>Londres</t>
         </is>
       </c>
-      <c r="B18" s="5" t="n">
+      <c r="B18" s="11" t="n">
         <v>1899</v>
       </c>
-      <c r="C18" s="5" t="n">
+      <c r="C18" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D18" s="5" t="n">
         <v>1797</v>
       </c>
-      <c r="E18" s="5" t="n">
+      <c r="E18" s="12" t="n">
         <v>0.9462875197472354</v>
       </c>
-      <c r="F18" s="5" t="n">
+      <c r="F18" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -4358,19 +4360,19 @@
           <t>Los Angeles (and vicinity), CA, US</t>
         </is>
       </c>
-      <c r="B19" s="5" t="n">
+      <c r="B19" s="11" t="n">
         <v>1838</v>
       </c>
-      <c r="C19" s="5" t="n">
+      <c r="C19" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D19" s="5" t="n">
         <v>1820</v>
       </c>
-      <c r="E19" s="5" t="n">
+      <c r="E19" s="12" t="n">
         <v>0.9902067464635473</v>
       </c>
-      <c r="F19" s="5" t="n">
+      <c r="F19" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G19" s="5" t="inlineStr">
@@ -4390,19 +4392,19 @@
           <t>El Cairo Area</t>
         </is>
       </c>
-      <c r="B20" s="5" t="n">
+      <c r="B20" s="11" t="n">
         <v>1491</v>
       </c>
-      <c r="C20" s="5" t="n">
+      <c r="C20" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D20" s="5" t="n">
         <v>1463</v>
       </c>
-      <c r="E20" s="5" t="n">
+      <c r="E20" s="12" t="n">
         <v>0.9812206572769953</v>
       </c>
-      <c r="F20" s="5" t="n">
+      <c r="F20" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -4422,19 +4424,19 @@
           <t>Miami Area</t>
         </is>
       </c>
-      <c r="B21" s="5" t="n">
+      <c r="B21" s="11" t="n">
         <v>1327</v>
       </c>
-      <c r="C21" s="5" t="n">
+      <c r="C21" s="11" t="n">
         <v>2</v>
       </c>
       <c r="D21" s="5" t="n">
         <v>1320</v>
       </c>
-      <c r="E21" s="5" t="n">
+      <c r="E21" s="12" t="n">
         <v>0.9947249434815373</v>
       </c>
-      <c r="F21" s="5" t="n">
+      <c r="F21" s="12" t="n">
         <v>0.001507159005275057</v>
       </c>
       <c r="G21" s="5" t="inlineStr">
@@ -4454,19 +4456,19 @@
           <t>Seattle Area</t>
         </is>
       </c>
-      <c r="B22" s="5" t="n">
+      <c r="B22" s="11" t="n">
         <v>1293</v>
       </c>
-      <c r="C22" s="5" t="n">
+      <c r="C22" s="11" t="n">
         <v>1</v>
       </c>
       <c r="D22" s="5" t="n">
         <v>1287</v>
       </c>
-      <c r="E22" s="5" t="n">
+      <c r="E22" s="12" t="n">
         <v>0.9953596287703016</v>
       </c>
-      <c r="F22" s="5" t="n">
+      <c r="F22" s="12" t="n">
         <v>0.0007733952049497294</v>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -4486,19 +4488,19 @@
           <t>Aruba</t>
         </is>
       </c>
-      <c r="B23" s="5" t="n">
+      <c r="B23" s="11" t="n">
         <v>1221</v>
       </c>
-      <c r="C23" s="5" t="n">
+      <c r="C23" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="5" t="n">
         <v>1218</v>
       </c>
-      <c r="E23" s="5" t="n">
+      <c r="E23" s="12" t="n">
         <v>0.9975429975429976</v>
       </c>
-      <c r="F23" s="5" t="n">
+      <c r="F23" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G23" s="5" t="inlineStr">
@@ -4518,19 +4520,19 @@
           <t>Hamburg Area</t>
         </is>
       </c>
-      <c r="B24" s="5" t="n">
+      <c r="B24" s="11" t="n">
         <v>1187</v>
       </c>
-      <c r="C24" s="5" t="n">
+      <c r="C24" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="5" t="n">
         <v>1181</v>
       </c>
-      <c r="E24" s="5" t="n">
+      <c r="E24" s="12" t="n">
         <v>0.9949452401010952</v>
       </c>
-      <c r="F24" s="5" t="n">
+      <c r="F24" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -4550,19 +4552,19 @@
           <t>Atlanta Area</t>
         </is>
       </c>
-      <c r="B25" s="5" t="n">
+      <c r="B25" s="11" t="n">
         <v>1142</v>
       </c>
-      <c r="C25" s="5" t="n">
+      <c r="C25" s="11" t="n">
         <v>1</v>
       </c>
       <c r="D25" s="5" t="n">
         <v>1127</v>
       </c>
-      <c r="E25" s="5" t="n">
+      <c r="E25" s="12" t="n">
         <v>0.9868651488616462</v>
       </c>
-      <c r="F25" s="5" t="n">
+      <c r="F25" s="12" t="n">
         <v>0.0008756567425569177</v>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -4582,19 +4584,19 @@
           <t>Denver (and vicinity), CO, US</t>
         </is>
       </c>
-      <c r="B26" s="5" t="n">
+      <c r="B26" s="11" t="n">
         <v>1092</v>
       </c>
-      <c r="C26" s="5" t="n">
+      <c r="C26" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="5" t="n">
         <v>1091</v>
       </c>
-      <c r="E26" s="5" t="n">
+      <c r="E26" s="12" t="n">
         <v>0.9990842490842491</v>
       </c>
-      <c r="F26" s="5" t="n">
+      <c r="F26" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -4614,19 +4616,19 @@
           <t>Budapest Area</t>
         </is>
       </c>
-      <c r="B27" s="5" t="n">
+      <c r="B27" s="11" t="n">
         <v>1017</v>
       </c>
-      <c r="C27" s="5" t="n">
+      <c r="C27" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="5" t="n">
         <v>996</v>
       </c>
-      <c r="E27" s="5" t="n">
+      <c r="E27" s="12" t="n">
         <v>0.9793510324483776</v>
       </c>
-      <c r="F27" s="5" t="n">
+      <c r="F27" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G27" s="5" t="inlineStr">
@@ -4646,19 +4648,19 @@
           <t>Acapulco</t>
         </is>
       </c>
-      <c r="B28" s="5" t="n">
+      <c r="B28" s="11" t="n">
         <v>1012</v>
       </c>
-      <c r="C28" s="5" t="n">
+      <c r="C28" s="11" t="n">
         <v>24</v>
       </c>
       <c r="D28" s="5" t="n">
         <v>862</v>
       </c>
-      <c r="E28" s="5" t="n">
+      <c r="E28" s="12" t="n">
         <v>0.8517786561264822</v>
       </c>
-      <c r="F28" s="5" t="n">
+      <c r="F28" s="12" t="n">
         <v>0.02371541501976284</v>
       </c>
       <c r="G28" s="5" t="inlineStr">
@@ -4678,19 +4680,19 @@
           <t>Malta Area</t>
         </is>
       </c>
-      <c r="B29" s="5" t="n">
+      <c r="B29" s="11" t="n">
         <v>1002</v>
       </c>
-      <c r="C29" s="5" t="n">
+      <c r="C29" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D29" s="5" t="n">
         <v>1002</v>
       </c>
-      <c r="E29" s="5" t="n">
+      <c r="E29" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F29" s="5" t="n">
+      <c r="F29" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G29" s="5" t="inlineStr">
@@ -4710,19 +4712,19 @@
           <t>Vancouver</t>
         </is>
       </c>
-      <c r="B30" s="5" t="n">
+      <c r="B30" s="11" t="n">
         <v>957</v>
       </c>
-      <c r="C30" s="5" t="n">
+      <c r="C30" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="5" t="n">
         <v>940</v>
       </c>
-      <c r="E30" s="5" t="n">
+      <c r="E30" s="12" t="n">
         <v>0.9822361546499477</v>
       </c>
-      <c r="F30" s="5" t="n">
+      <c r="F30" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G30" s="5" t="inlineStr">
@@ -4742,19 +4744,19 @@
           <t>Ixtapa / Zihuatanejo</t>
         </is>
       </c>
-      <c r="B31" s="5" t="n">
+      <c r="B31" s="11" t="n">
         <v>931</v>
       </c>
-      <c r="C31" s="5" t="n">
+      <c r="C31" s="11" t="n">
         <v>5</v>
       </c>
       <c r="D31" s="5" t="n">
         <v>426</v>
       </c>
-      <c r="E31" s="5" t="n">
+      <c r="E31" s="12" t="n">
         <v>0.4575725026852847</v>
       </c>
-      <c r="F31" s="5" t="n">
+      <c r="F31" s="12" t="n">
         <v>0.005370569280343717</v>
       </c>
       <c r="G31" s="5" t="inlineStr">
@@ -4774,19 +4776,19 @@
           <t>French Riviera Area</t>
         </is>
       </c>
-      <c r="B32" s="5" t="n">
+      <c r="B32" s="11" t="n">
         <v>842</v>
       </c>
-      <c r="C32" s="5" t="n">
+      <c r="C32" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="5" t="n">
         <v>825</v>
       </c>
-      <c r="E32" s="5" t="n">
+      <c r="E32" s="12" t="n">
         <v>0.9798099762470309</v>
       </c>
-      <c r="F32" s="5" t="n">
+      <c r="F32" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G32" s="5" t="inlineStr">
@@ -4806,19 +4808,19 @@
           <t>Cartagena Area</t>
         </is>
       </c>
-      <c r="B33" s="5" t="n">
+      <c r="B33" s="11" t="n">
         <v>825</v>
       </c>
-      <c r="C33" s="5" t="n">
+      <c r="C33" s="11" t="n">
         <v>1</v>
       </c>
       <c r="D33" s="5" t="n">
         <v>454</v>
       </c>
-      <c r="E33" s="5" t="n">
+      <c r="E33" s="12" t="n">
         <v>0.5503030303030303</v>
       </c>
-      <c r="F33" s="5" t="n">
+      <c r="F33" s="12" t="n">
         <v>0.001212121212121212</v>
       </c>
       <c r="G33" s="5" t="inlineStr">
@@ -4838,19 +4840,19 @@
           <t>Puerto Rico</t>
         </is>
       </c>
-      <c r="B34" s="5" t="n">
+      <c r="B34" s="11" t="n">
         <v>812</v>
       </c>
-      <c r="C34" s="5" t="n">
+      <c r="C34" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="5" t="n">
         <v>805</v>
       </c>
-      <c r="E34" s="5" t="n">
+      <c r="E34" s="12" t="n">
         <v>0.9913793103448276</v>
       </c>
-      <c r="F34" s="5" t="n">
+      <c r="F34" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G34" s="5" t="inlineStr">
@@ -4870,19 +4872,19 @@
           <t>Puerto Vallarta Area</t>
         </is>
       </c>
-      <c r="B35" s="5" t="n">
+      <c r="B35" s="11" t="n">
         <v>811</v>
       </c>
-      <c r="C35" s="5" t="n">
+      <c r="C35" s="11" t="n">
         <v>10</v>
       </c>
       <c r="D35" s="5" t="n">
         <v>811</v>
       </c>
-      <c r="E35" s="5" t="n">
+      <c r="E35" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F35" s="5" t="n">
+      <c r="F35" s="12" t="n">
         <v>0.01233045622688039</v>
       </c>
       <c r="G35" s="5" t="inlineStr">
@@ -4902,19 +4904,19 @@
           <t>Dallas</t>
         </is>
       </c>
-      <c r="B36" s="5" t="n">
+      <c r="B36" s="11" t="n">
         <v>795</v>
       </c>
-      <c r="C36" s="5" t="n">
+      <c r="C36" s="11" t="n">
         <v>2</v>
       </c>
       <c r="D36" s="5" t="n">
         <v>774</v>
       </c>
-      <c r="E36" s="5" t="n">
+      <c r="E36" s="12" t="n">
         <v>0.9735849056603774</v>
       </c>
-      <c r="F36" s="5" t="n">
+      <c r="F36" s="12" t="n">
         <v>0.002515723270440251</v>
       </c>
       <c r="G36" s="5" t="inlineStr">
@@ -4934,19 +4936,19 @@
           <t>Vienna Area</t>
         </is>
       </c>
-      <c r="B37" s="5" t="n">
+      <c r="B37" s="11" t="n">
         <v>762</v>
       </c>
-      <c r="C37" s="5" t="n">
+      <c r="C37" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="5" t="n">
         <v>755</v>
       </c>
-      <c r="E37" s="5" t="n">
+      <c r="E37" s="12" t="n">
         <v>0.9908136482939632</v>
       </c>
-      <c r="F37" s="5" t="n">
+      <c r="F37" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G37" s="5" t="inlineStr">
@@ -4966,19 +4968,19 @@
           <t>Punta Cana</t>
         </is>
       </c>
-      <c r="B38" s="5" t="n">
+      <c r="B38" s="11" t="n">
         <v>760</v>
       </c>
-      <c r="C38" s="5" t="n">
+      <c r="C38" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D38" s="5" t="n">
         <v>758</v>
       </c>
-      <c r="E38" s="5" t="n">
+      <c r="E38" s="12" t="n">
         <v>0.9973684210526316</v>
       </c>
-      <c r="F38" s="5" t="n">
+      <c r="F38" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G38" s="5" t="inlineStr">
@@ -4998,19 +5000,19 @@
           <t>Mexico City - Central Mexico</t>
         </is>
       </c>
-      <c r="B39" s="5" t="n">
+      <c r="B39" s="11" t="n">
         <v>736</v>
       </c>
-      <c r="C39" s="5" t="n">
+      <c r="C39" s="11" t="n">
         <v>40</v>
       </c>
       <c r="D39" s="5" t="n">
         <v>732</v>
       </c>
-      <c r="E39" s="5" t="n">
+      <c r="E39" s="12" t="n">
         <v>0.9945652173913043</v>
       </c>
-      <c r="F39" s="5" t="n">
+      <c r="F39" s="12" t="n">
         <v>0.05434782608695652</v>
       </c>
       <c r="G39" s="5" t="inlineStr">
@@ -5030,19 +5032,19 @@
           <t>Montreal</t>
         </is>
       </c>
-      <c r="B40" s="5" t="n">
+      <c r="B40" s="11" t="n">
         <v>728</v>
       </c>
-      <c r="C40" s="5" t="n">
+      <c r="C40" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D40" s="5" t="n">
         <v>720</v>
       </c>
-      <c r="E40" s="5" t="n">
+      <c r="E40" s="12" t="n">
         <v>0.9890109890109891</v>
       </c>
-      <c r="F40" s="5" t="n">
+      <c r="F40" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G40" s="5" t="inlineStr">
@@ -5062,19 +5064,19 @@
           <t>San Francisco</t>
         </is>
       </c>
-      <c r="B41" s="5" t="n">
+      <c r="B41" s="11" t="n">
         <v>699</v>
       </c>
-      <c r="C41" s="5" t="n">
+      <c r="C41" s="11" t="n">
         <v>1</v>
       </c>
       <c r="D41" s="5" t="n">
         <v>488</v>
       </c>
-      <c r="E41" s="5" t="n">
+      <c r="E41" s="12" t="n">
         <v>0.698140200286123</v>
       </c>
-      <c r="F41" s="5" t="n">
+      <c r="F41" s="12" t="n">
         <v>0.001430615164520744</v>
       </c>
       <c r="G41" s="5" t="inlineStr">
@@ -5094,19 +5096,19 @@
           <t>Riviera Nayarit</t>
         </is>
       </c>
-      <c r="B42" s="5" t="n">
+      <c r="B42" s="11" t="n">
         <v>668</v>
       </c>
-      <c r="C42" s="5" t="n">
+      <c r="C42" s="11" t="n">
         <v>7</v>
       </c>
       <c r="D42" s="5" t="n">
         <v>641</v>
       </c>
-      <c r="E42" s="5" t="n">
+      <c r="E42" s="12" t="n">
         <v>0.9595808383233533</v>
       </c>
-      <c r="F42" s="5" t="n">
+      <c r="F42" s="12" t="n">
         <v>0.01047904191616766</v>
       </c>
       <c r="G42" s="5" t="inlineStr">
@@ -5126,19 +5128,19 @@
           <t>Greenville Area</t>
         </is>
       </c>
-      <c r="B43" s="5" t="n">
+      <c r="B43" s="11" t="n">
         <v>648</v>
       </c>
-      <c r="C43" s="5" t="n">
+      <c r="C43" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D43" s="5" t="n">
         <v>568</v>
       </c>
-      <c r="E43" s="5" t="n">
+      <c r="E43" s="12" t="n">
         <v>0.8765432098765432</v>
       </c>
-      <c r="F43" s="5" t="n">
+      <c r="F43" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G43" s="5" t="inlineStr">
@@ -5158,19 +5160,19 @@
           <t>Amsterdam</t>
         </is>
       </c>
-      <c r="B44" s="5" t="n">
+      <c r="B44" s="11" t="n">
         <v>647</v>
       </c>
-      <c r="C44" s="5" t="n">
+      <c r="C44" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D44" s="5" t="n">
         <v>642</v>
       </c>
-      <c r="E44" s="5" t="n">
+      <c r="E44" s="12" t="n">
         <v>0.9922720247295209</v>
       </c>
-      <c r="F44" s="5" t="n">
+      <c r="F44" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G44" s="5" t="inlineStr">
@@ -5190,19 +5192,19 @@
           <t>Monterrey</t>
         </is>
       </c>
-      <c r="B45" s="5" t="n">
+      <c r="B45" s="11" t="n">
         <v>634</v>
       </c>
-      <c r="C45" s="5" t="n">
+      <c r="C45" s="11" t="n">
         <v>67</v>
       </c>
       <c r="D45" s="5" t="n">
         <v>471</v>
       </c>
-      <c r="E45" s="5" t="n">
+      <c r="E45" s="12" t="n">
         <v>0.7429022082018928</v>
       </c>
-      <c r="F45" s="5" t="n">
+      <c r="F45" s="12" t="n">
         <v>0.1056782334384858</v>
       </c>
       <c r="G45" s="5" t="inlineStr">
@@ -5222,19 +5224,19 @@
           <t>Barcelona</t>
         </is>
       </c>
-      <c r="B46" s="5" t="n">
+      <c r="B46" s="11" t="n">
         <v>620</v>
       </c>
-      <c r="C46" s="5" t="n">
+      <c r="C46" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D46" s="5" t="n">
         <v>563</v>
       </c>
-      <c r="E46" s="5" t="n">
+      <c r="E46" s="12" t="n">
         <v>0.9080645161290323</v>
       </c>
-      <c r="F46" s="5" t="n">
+      <c r="F46" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G46" s="5" t="inlineStr">
@@ -5254,19 +5256,19 @@
           <t>San Antonio</t>
         </is>
       </c>
-      <c r="B47" s="5" t="n">
+      <c r="B47" s="11" t="n">
         <v>559</v>
       </c>
-      <c r="C47" s="5" t="n">
+      <c r="C47" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D47" s="5" t="n">
         <v>552</v>
       </c>
-      <c r="E47" s="5" t="n">
+      <c r="E47" s="12" t="n">
         <v>0.9874776386404294</v>
       </c>
-      <c r="F47" s="5" t="n">
+      <c r="F47" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G47" s="5" t="inlineStr">
@@ -5286,19 +5288,19 @@
           <t>Austin</t>
         </is>
       </c>
-      <c r="B48" s="5" t="n">
+      <c r="B48" s="11" t="n">
         <v>513</v>
       </c>
-      <c r="C48" s="5" t="n">
+      <c r="C48" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D48" s="5" t="n">
         <v>495</v>
       </c>
-      <c r="E48" s="5" t="n">
+      <c r="E48" s="12" t="n">
         <v>0.9649122807017544</v>
       </c>
-      <c r="F48" s="5" t="n">
+      <c r="F48" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G48" s="5" t="inlineStr">
@@ -5318,19 +5320,19 @@
           <t>Anaheim Area</t>
         </is>
       </c>
-      <c r="B49" s="5" t="n">
+      <c r="B49" s="11" t="n">
         <v>504</v>
       </c>
-      <c r="C49" s="5" t="n">
+      <c r="C49" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D49" s="5" t="n">
         <v>501</v>
       </c>
-      <c r="E49" s="5" t="n">
+      <c r="E49" s="12" t="n">
         <v>0.9940476190476191</v>
       </c>
-      <c r="F49" s="5" t="n">
+      <c r="F49" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G49" s="5" t="inlineStr">
@@ -5350,19 +5352,19 @@
           <t>Munich Area</t>
         </is>
       </c>
-      <c r="B50" s="5" t="n">
+      <c r="B50" s="11" t="n">
         <v>483</v>
       </c>
-      <c r="C50" s="5" t="n">
+      <c r="C50" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D50" s="5" t="n">
         <v>479</v>
       </c>
-      <c r="E50" s="5" t="n">
+      <c r="E50" s="12" t="n">
         <v>0.9917184265010351</v>
       </c>
-      <c r="F50" s="5" t="n">
+      <c r="F50" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G50" s="5" t="inlineStr">
@@ -5382,19 +5384,19 @@
           <t>Fort Lauderdale (and vicinity), FL, US</t>
         </is>
       </c>
-      <c r="B51" s="5" t="n">
+      <c r="B51" s="11" t="n">
         <v>476</v>
       </c>
-      <c r="C51" s="5" t="n">
+      <c r="C51" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D51" s="5" t="n">
         <v>476</v>
       </c>
-      <c r="E51" s="5" t="n">
+      <c r="E51" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F51" s="5" t="n">
+      <c r="F51" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G51" s="5" t="inlineStr">
@@ -5414,19 +5416,19 @@
           <t>London Area</t>
         </is>
       </c>
-      <c r="B52" s="5" t="n">
+      <c r="B52" s="11" t="n">
         <v>467</v>
       </c>
-      <c r="C52" s="5" t="n">
+      <c r="C52" s="11" t="n">
         <v>6</v>
       </c>
       <c r="D52" s="5" t="n">
         <v>460</v>
       </c>
-      <c r="E52" s="5" t="n">
+      <c r="E52" s="12" t="n">
         <v>0.9850107066381156</v>
       </c>
-      <c r="F52" s="5" t="n">
+      <c r="F52" s="12" t="n">
         <v>0.01284796573875803</v>
       </c>
       <c r="G52" s="5" t="inlineStr">
@@ -5446,19 +5448,19 @@
           <t>São Paulo</t>
         </is>
       </c>
-      <c r="B53" s="5" t="n">
+      <c r="B53" s="11" t="n">
         <v>442</v>
       </c>
-      <c r="C53" s="5" t="n">
+      <c r="C53" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D53" s="5" t="n">
         <v>385</v>
       </c>
-      <c r="E53" s="5" t="n">
+      <c r="E53" s="12" t="n">
         <v>0.8710407239819005</v>
       </c>
-      <c r="F53" s="5" t="n">
+      <c r="F53" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G53" s="5" t="inlineStr">
@@ -5478,19 +5480,19 @@
           <t>Clearwater</t>
         </is>
       </c>
-      <c r="B54" s="5" t="n">
+      <c r="B54" s="11" t="n">
         <v>393</v>
       </c>
-      <c r="C54" s="5" t="n">
+      <c r="C54" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D54" s="5" t="n">
         <v>393</v>
       </c>
-      <c r="E54" s="5" t="n">
+      <c r="E54" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F54" s="5" t="n">
+      <c r="F54" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G54" s="5" t="inlineStr">
@@ -5510,19 +5512,19 @@
           <t>Abu Dhabi</t>
         </is>
       </c>
-      <c r="B55" s="5" t="n">
+      <c r="B55" s="11" t="n">
         <v>380</v>
       </c>
-      <c r="C55" s="5" t="n">
+      <c r="C55" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D55" s="5" t="n">
         <v>380</v>
       </c>
-      <c r="E55" s="5" t="n">
+      <c r="E55" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F55" s="5" t="n">
+      <c r="F55" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G55" s="5" t="inlineStr">
@@ -5542,19 +5544,19 @@
           <t>Nashville (and vicinity), TN, US</t>
         </is>
       </c>
-      <c r="B56" s="5" t="n">
+      <c r="B56" s="11" t="n">
         <v>365</v>
       </c>
-      <c r="C56" s="5" t="n">
+      <c r="C56" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D56" s="5" t="n">
         <v>365</v>
       </c>
-      <c r="E56" s="5" t="n">
+      <c r="E56" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F56" s="5" t="n">
+      <c r="F56" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G56" s="5" t="inlineStr">
@@ -5574,19 +5576,19 @@
           <t>San Diego</t>
         </is>
       </c>
-      <c r="B57" s="5" t="n">
+      <c r="B57" s="11" t="n">
         <v>365</v>
       </c>
-      <c r="C57" s="5" t="n">
+      <c r="C57" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D57" s="5" t="n">
         <v>357</v>
       </c>
-      <c r="E57" s="5" t="n">
+      <c r="E57" s="12" t="n">
         <v>0.9780821917808219</v>
       </c>
-      <c r="F57" s="5" t="n">
+      <c r="F57" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G57" s="5" t="inlineStr">
@@ -5606,19 +5608,19 @@
           <t>Laughlin Area</t>
         </is>
       </c>
-      <c r="B58" s="5" t="n">
+      <c r="B58" s="11" t="n">
         <v>364</v>
       </c>
-      <c r="C58" s="5" t="n">
+      <c r="C58" s="11" t="n">
         <v>13</v>
       </c>
       <c r="D58" s="5" t="n">
         <v>319</v>
       </c>
-      <c r="E58" s="5" t="n">
+      <c r="E58" s="12" t="n">
         <v>0.8763736263736264</v>
       </c>
-      <c r="F58" s="5" t="n">
+      <c r="F58" s="12" t="n">
         <v>0.03571428571428571</v>
       </c>
       <c r="G58" s="5" t="inlineStr">
@@ -5638,19 +5640,19 @@
           <t>Jamaica</t>
         </is>
       </c>
-      <c r="B59" s="5" t="n">
+      <c r="B59" s="11" t="n">
         <v>351</v>
       </c>
-      <c r="C59" s="5" t="n">
+      <c r="C59" s="11" t="n">
         <v>1</v>
       </c>
       <c r="D59" s="5" t="n">
         <v>350</v>
       </c>
-      <c r="E59" s="5" t="n">
+      <c r="E59" s="12" t="n">
         <v>0.9971509971509972</v>
       </c>
-      <c r="F59" s="5" t="n">
+      <c r="F59" s="12" t="n">
         <v>0.002849002849002849</v>
       </c>
       <c r="G59" s="5" t="inlineStr">
@@ -5670,19 +5672,19 @@
           <t>Medellin Area</t>
         </is>
       </c>
-      <c r="B60" s="5" t="n">
+      <c r="B60" s="11" t="n">
         <v>323</v>
       </c>
-      <c r="C60" s="5" t="n">
+      <c r="C60" s="11" t="n">
         <v>2</v>
       </c>
       <c r="D60" s="5" t="n">
         <v>318</v>
       </c>
-      <c r="E60" s="5" t="n">
+      <c r="E60" s="12" t="n">
         <v>0.9845201238390093</v>
       </c>
-      <c r="F60" s="5" t="n">
+      <c r="F60" s="12" t="n">
         <v>0.006191950464396285</v>
       </c>
       <c r="G60" s="5" t="inlineStr">
@@ -5702,19 +5704,19 @@
           <t>Monterey Area</t>
         </is>
       </c>
-      <c r="B61" s="5" t="n">
+      <c r="B61" s="11" t="n">
         <v>312</v>
       </c>
-      <c r="C61" s="5" t="n">
+      <c r="C61" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D61" s="5" t="n">
         <v>312</v>
       </c>
-      <c r="E61" s="5" t="n">
+      <c r="E61" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F61" s="5" t="n">
+      <c r="F61" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G61" s="5" t="inlineStr">
@@ -5734,19 +5736,19 @@
           <t>Provence Area</t>
         </is>
       </c>
-      <c r="B62" s="5" t="n">
+      <c r="B62" s="11" t="n">
         <v>304</v>
       </c>
-      <c r="C62" s="5" t="n">
+      <c r="C62" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D62" s="5" t="n">
         <v>304</v>
       </c>
-      <c r="E62" s="5" t="n">
+      <c r="E62" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F62" s="5" t="n">
+      <c r="F62" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G62" s="5" t="inlineStr">
@@ -5766,19 +5768,19 @@
           <t>Atenas</t>
         </is>
       </c>
-      <c r="B63" s="5" t="n">
+      <c r="B63" s="11" t="n">
         <v>271</v>
       </c>
-      <c r="C63" s="5" t="n">
+      <c r="C63" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D63" s="5" t="n">
         <v>250</v>
       </c>
-      <c r="E63" s="5" t="n">
+      <c r="E63" s="12" t="n">
         <v>0.922509225092251</v>
       </c>
-      <c r="F63" s="5" t="n">
+      <c r="F63" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G63" s="5" t="inlineStr">
@@ -5798,19 +5800,19 @@
           <t>Bogotá Area</t>
         </is>
       </c>
-      <c r="B64" s="5" t="n">
+      <c r="B64" s="11" t="n">
         <v>234</v>
       </c>
-      <c r="C64" s="5" t="n">
+      <c r="C64" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D64" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="E64" s="5" t="n">
+      <c r="E64" s="12" t="n">
         <v>0.06837606837606838</v>
       </c>
-      <c r="F64" s="5" t="n">
+      <c r="F64" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G64" s="5" t="inlineStr">
@@ -5830,19 +5832,19 @@
           <t>Milan</t>
         </is>
       </c>
-      <c r="B65" s="5" t="n">
+      <c r="B65" s="11" t="n">
         <v>233</v>
       </c>
-      <c r="C65" s="5" t="n">
+      <c r="C65" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D65" s="5" t="n">
         <v>232</v>
       </c>
-      <c r="E65" s="5" t="n">
+      <c r="E65" s="12" t="n">
         <v>0.9957081545064378</v>
       </c>
-      <c r="F65" s="5" t="n">
+      <c r="F65" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G65" s="5" t="inlineStr">
@@ -5862,19 +5864,19 @@
           <t>La Romana Area</t>
         </is>
       </c>
-      <c r="B66" s="5" t="n">
+      <c r="B66" s="11" t="n">
         <v>229</v>
       </c>
-      <c r="C66" s="5" t="n">
+      <c r="C66" s="11" t="n">
         <v>3</v>
       </c>
       <c r="D66" s="5" t="n">
         <v>229</v>
       </c>
-      <c r="E66" s="5" t="n">
+      <c r="E66" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F66" s="5" t="n">
+      <c r="F66" s="12" t="n">
         <v>0.01310043668122271</v>
       </c>
       <c r="G66" s="5" t="inlineStr">
@@ -5894,19 +5896,19 @@
           <t>Phoenix (and vicinity), AZ, US</t>
         </is>
       </c>
-      <c r="B67" s="5" t="n">
+      <c r="B67" s="11" t="n">
         <v>224</v>
       </c>
-      <c r="C67" s="5" t="n">
+      <c r="C67" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D67" s="5" t="n">
         <v>182</v>
       </c>
-      <c r="E67" s="5" t="n">
+      <c r="E67" s="12" t="n">
         <v>0.8125</v>
       </c>
-      <c r="F67" s="5" t="n">
+      <c r="F67" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G67" s="5" t="inlineStr">
@@ -5926,19 +5928,19 @@
           <t>Sheridan Area</t>
         </is>
       </c>
-      <c r="B68" s="5" t="n">
+      <c r="B68" s="11" t="n">
         <v>221</v>
       </c>
-      <c r="C68" s="5" t="n">
+      <c r="C68" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D68" s="5" t="n">
         <v>221</v>
       </c>
-      <c r="E68" s="5" t="n">
+      <c r="E68" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F68" s="5" t="n">
+      <c r="F68" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G68" s="5" t="inlineStr">
@@ -5958,19 +5960,19 @@
           <t>Space Coast Area</t>
         </is>
       </c>
-      <c r="B69" s="5" t="n">
+      <c r="B69" s="11" t="n">
         <v>212</v>
       </c>
-      <c r="C69" s="5" t="n">
+      <c r="C69" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D69" s="5" t="n">
         <v>212</v>
       </c>
-      <c r="E69" s="5" t="n">
+      <c r="E69" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F69" s="5" t="n">
+      <c r="F69" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G69" s="5" t="inlineStr">
@@ -5990,19 +5992,19 @@
           <t>Río de Janeiro</t>
         </is>
       </c>
-      <c r="B70" s="5" t="n">
+      <c r="B70" s="11" t="n">
         <v>210</v>
       </c>
-      <c r="C70" s="5" t="n">
+      <c r="C70" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D70" s="5" t="n">
         <v>210</v>
       </c>
-      <c r="E70" s="5" t="n">
+      <c r="E70" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F70" s="5" t="n">
+      <c r="F70" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G70" s="5" t="inlineStr">
@@ -6022,19 +6024,19 @@
           <t>Múnich Area</t>
         </is>
       </c>
-      <c r="B71" s="5" t="n">
+      <c r="B71" s="11" t="n">
         <v>203</v>
       </c>
-      <c r="C71" s="5" t="n">
+      <c r="C71" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D71" s="5" t="n">
         <v>200</v>
       </c>
-      <c r="E71" s="5" t="n">
+      <c r="E71" s="12" t="n">
         <v>0.9852216748768473</v>
       </c>
-      <c r="F71" s="5" t="n">
+      <c r="F71" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G71" s="5" t="inlineStr">
@@ -6054,19 +6056,19 @@
           <t>Veneto Area</t>
         </is>
       </c>
-      <c r="B72" s="5" t="n">
+      <c r="B72" s="11" t="n">
         <v>201</v>
       </c>
-      <c r="C72" s="5" t="n">
+      <c r="C72" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D72" s="5" t="n">
         <v>196</v>
       </c>
-      <c r="E72" s="5" t="n">
+      <c r="E72" s="12" t="n">
         <v>0.9751243781094527</v>
       </c>
-      <c r="F72" s="5" t="n">
+      <c r="F72" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G72" s="5" t="inlineStr">
@@ -6086,19 +6088,19 @@
           <t>Omaha Area</t>
         </is>
       </c>
-      <c r="B73" s="5" t="n">
+      <c r="B73" s="11" t="n">
         <v>198</v>
       </c>
-      <c r="C73" s="5" t="n">
+      <c r="C73" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D73" s="5" t="n">
         <v>196</v>
       </c>
-      <c r="E73" s="5" t="n">
+      <c r="E73" s="12" t="n">
         <v>0.9898989898989899</v>
       </c>
-      <c r="F73" s="5" t="n">
+      <c r="F73" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G73" s="5" t="inlineStr">
@@ -6118,19 +6120,19 @@
           <t>Madrid</t>
         </is>
       </c>
-      <c r="B74" s="5" t="n">
+      <c r="B74" s="11" t="n">
         <v>191</v>
       </c>
-      <c r="C74" s="5" t="n">
+      <c r="C74" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D74" s="5" t="n">
         <v>191</v>
       </c>
-      <c r="E74" s="5" t="n">
+      <c r="E74" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F74" s="5" t="n">
+      <c r="F74" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G74" s="5" t="inlineStr">
@@ -6150,19 +6152,19 @@
           <t>Hawái</t>
         </is>
       </c>
-      <c r="B75" s="5" t="n">
+      <c r="B75" s="11" t="n">
         <v>191</v>
       </c>
-      <c r="C75" s="5" t="n">
+      <c r="C75" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D75" s="5" t="n">
         <v>191</v>
       </c>
-      <c r="E75" s="5" t="n">
+      <c r="E75" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F75" s="5" t="n">
+      <c r="F75" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G75" s="5" t="inlineStr">
@@ -6182,19 +6184,19 @@
           <t>New Orleans</t>
         </is>
       </c>
-      <c r="B76" s="5" t="n">
+      <c r="B76" s="11" t="n">
         <v>190</v>
       </c>
-      <c r="C76" s="5" t="n">
+      <c r="C76" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D76" s="5" t="n">
         <v>189</v>
       </c>
-      <c r="E76" s="5" t="n">
+      <c r="E76" s="12" t="n">
         <v>0.9947368421052631</v>
       </c>
-      <c r="F76" s="5" t="n">
+      <c r="F76" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G76" s="5" t="inlineStr">
@@ -6214,19 +6216,19 @@
           <t>Minneapolis - St. Paul Area</t>
         </is>
       </c>
-      <c r="B77" s="5" t="n">
+      <c r="B77" s="11" t="n">
         <v>189</v>
       </c>
-      <c r="C77" s="5" t="n">
+      <c r="C77" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="5" t="n">
         <v>188</v>
       </c>
-      <c r="E77" s="5" t="n">
+      <c r="E77" s="12" t="n">
         <v>0.9947089947089947</v>
       </c>
-      <c r="F77" s="5" t="n">
+      <c r="F77" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G77" s="5" t="inlineStr">
@@ -6246,19 +6248,19 @@
           <t>Merida</t>
         </is>
       </c>
-      <c r="B78" s="5" t="n">
+      <c r="B78" s="11" t="n">
         <v>187</v>
       </c>
-      <c r="C78" s="5" t="n">
+      <c r="C78" s="11" t="n">
         <v>14</v>
       </c>
       <c r="D78" s="5" t="n">
         <v>187</v>
       </c>
-      <c r="E78" s="5" t="n">
+      <c r="E78" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F78" s="5" t="n">
+      <c r="F78" s="12" t="n">
         <v>0.0748663101604278</v>
       </c>
       <c r="G78" s="5" t="inlineStr">
@@ -6278,19 +6280,19 @@
           <t>Grand Canyon</t>
         </is>
       </c>
-      <c r="B79" s="5" t="n">
+      <c r="B79" s="11" t="n">
         <v>182</v>
       </c>
-      <c r="C79" s="5" t="n">
+      <c r="C79" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D79" s="5" t="n">
         <v>169</v>
       </c>
-      <c r="E79" s="5" t="n">
+      <c r="E79" s="12" t="n">
         <v>0.9285714285714286</v>
       </c>
-      <c r="F79" s="5" t="n">
+      <c r="F79" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G79" s="5" t="inlineStr">
@@ -6310,19 +6312,19 @@
           <t>Cleveland Area</t>
         </is>
       </c>
-      <c r="B80" s="5" t="n">
+      <c r="B80" s="11" t="n">
         <v>178</v>
       </c>
-      <c r="C80" s="5" t="n">
+      <c r="C80" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D80" s="5" t="n">
         <v>172</v>
       </c>
-      <c r="E80" s="5" t="n">
+      <c r="E80" s="12" t="n">
         <v>0.9662921348314607</v>
       </c>
-      <c r="F80" s="5" t="n">
+      <c r="F80" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G80" s="5" t="inlineStr">
@@ -6342,19 +6344,19 @@
           <t>Istanbul Area</t>
         </is>
       </c>
-      <c r="B81" s="5" t="n">
+      <c r="B81" s="11" t="n">
         <v>177</v>
       </c>
-      <c r="C81" s="5" t="n">
+      <c r="C81" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D81" s="5" t="n">
         <v>177</v>
       </c>
-      <c r="E81" s="5" t="n">
+      <c r="E81" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F81" s="5" t="n">
+      <c r="F81" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G81" s="5" t="inlineStr">
@@ -6374,19 +6376,19 @@
           <t>Salt Lake City Area</t>
         </is>
       </c>
-      <c r="B82" s="5" t="n">
+      <c r="B82" s="11" t="n">
         <v>177</v>
       </c>
-      <c r="C82" s="5" t="n">
+      <c r="C82" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D82" s="5" t="n">
         <v>174</v>
       </c>
-      <c r="E82" s="5" t="n">
+      <c r="E82" s="12" t="n">
         <v>0.9830508474576272</v>
       </c>
-      <c r="F82" s="5" t="n">
+      <c r="F82" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G82" s="5" t="inlineStr">
@@ -6406,19 +6408,19 @@
           <t>Rome Area</t>
         </is>
       </c>
-      <c r="B83" s="5" t="n">
+      <c r="B83" s="11" t="n">
         <v>166</v>
       </c>
-      <c r="C83" s="5" t="n">
+      <c r="C83" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D83" s="5" t="n">
         <v>166</v>
       </c>
-      <c r="E83" s="5" t="n">
+      <c r="E83" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F83" s="5" t="n">
+      <c r="F83" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G83" s="5" t="inlineStr">
@@ -6438,19 +6440,19 @@
           <t>Ottawa Area</t>
         </is>
       </c>
-      <c r="B84" s="5" t="n">
+      <c r="B84" s="11" t="n">
         <v>166</v>
       </c>
-      <c r="C84" s="5" t="n">
+      <c r="C84" s="11" t="n">
         <v>10</v>
       </c>
       <c r="D84" s="5" t="n">
         <v>164</v>
       </c>
-      <c r="E84" s="5" t="n">
+      <c r="E84" s="12" t="n">
         <v>0.9879518072289156</v>
       </c>
-      <c r="F84" s="5" t="n">
+      <c r="F84" s="12" t="n">
         <v>0.06024096385542169</v>
       </c>
       <c r="G84" s="5" t="inlineStr">
@@ -6470,19 +6472,19 @@
           <t>Algarve Area</t>
         </is>
       </c>
-      <c r="B85" s="5" t="n">
+      <c r="B85" s="11" t="n">
         <v>154</v>
       </c>
-      <c r="C85" s="5" t="n">
+      <c r="C85" s="11" t="n">
         <v>1</v>
       </c>
       <c r="D85" s="5" t="n">
         <v>154</v>
       </c>
-      <c r="E85" s="5" t="n">
+      <c r="E85" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F85" s="5" t="n">
+      <c r="F85" s="12" t="n">
         <v>0.006493506493506494</v>
       </c>
       <c r="G85" s="5" t="inlineStr">
@@ -6502,19 +6504,19 @@
           <t>San Luis, Misuri Area</t>
         </is>
       </c>
-      <c r="B86" s="5" t="n">
+      <c r="B86" s="11" t="n">
         <v>154</v>
       </c>
-      <c r="C86" s="5" t="n">
+      <c r="C86" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D86" s="5" t="n">
         <v>151</v>
       </c>
-      <c r="E86" s="5" t="n">
+      <c r="E86" s="12" t="n">
         <v>0.9805194805194806</v>
       </c>
-      <c r="F86" s="5" t="n">
+      <c r="F86" s="12" t="n">
         <v>0</v>
       </c>
       <c r="G86" s="5" t="inlineStr">
@@ -6534,19 +6536,19 @@
           <t>Puerto Escondido Area</t>
         </is>
       </c>
-      <c r="B87" s="5" t="n">
+      <c r="B87" s="11" t="n">
         <v>153</v>
       </c>
-      <c r="C87" s="5" t="n">
+      <c r="C87" s="11" t="n">
         <v>13</v>
       </c>
       <c r="D87" s="5" t="n">
         <v>124</v>
       </c>
-      <c r="E87" s="5" t="n">
+      <c r="E87" s="12" t="n">
         <v>0.8104575163398693</v>
       </c>
-      <c r="F87" s="5" t="n">
+      <c r="F87" s="12" t="n">
         <v>0.08496732026143791</v>
       </c>
       <c r="G87" s="5" t="inlineStr">
@@ -6594,7 +6596,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:52 · W21 · 18–24 may 2026</t>
+          <t>Generado: 25/05/2026 23:40 · W21 · 18–24 may 2026</t>
         </is>
       </c>
     </row>
@@ -6646,19 +6648,19 @@
           <t>DerbySoft</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="11" t="n">
         <v>75843</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="11" t="n">
         <v>55</v>
       </c>
       <c r="D6" s="5" t="n">
         <v>73544</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="12" t="n">
         <v>0.9696873805097372</v>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="F6" s="12" t="n">
         <v>0.0007251822844560474</v>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -6678,19 +6680,19 @@
           <t>HBSI</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B7" s="11" t="n">
         <v>16922</v>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="11" t="n">
         <v>57</v>
       </c>
       <c r="D7" s="5" t="n">
         <v>11650</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="12" t="n">
         <v>0.6884529015482803</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" s="12" t="n">
         <v>0.003368396170665406</v>
       </c>
       <c r="G7" s="5" t="inlineStr">
@@ -6710,19 +6712,19 @@
           <t>Internal</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="11" t="n">
         <v>13846</v>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="11" t="n">
         <v>195</v>
       </c>
       <c r="D8" s="5" t="n">
         <v>11643</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="12" t="n">
         <v>0.8408926765852954</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F8" s="12" t="n">
         <v>0.01408348981655352</v>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -6742,19 +6744,19 @@
           <t>SynXis</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="11" t="n">
         <v>978</v>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="11" t="n">
         <v>7</v>
       </c>
       <c r="D9" s="5" t="n">
         <v>838</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="12" t="n">
         <v>0.8568507157464212</v>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="F9" s="12" t="n">
         <v>0.007157464212678937</v>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -6774,19 +6776,19 @@
           <t>Travelclick</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" s="11" t="n">
         <v>695</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="11" t="n">
         <v>85</v>
       </c>
       <c r="D10" s="5" t="n">
         <v>695</v>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E10" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F10" s="5" t="n">
+      <c r="F10" s="12" t="n">
         <v>0.1223021582733813</v>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -6806,19 +6808,19 @@
           <t>Siteminder</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n">
+      <c r="B11" s="11" t="n">
         <v>489</v>
       </c>
-      <c r="C11" s="5" t="n">
+      <c r="C11" s="11" t="n">
         <v>4</v>
       </c>
       <c r="D11" s="5" t="n">
         <v>489</v>
       </c>
-      <c r="E11" s="5" t="n">
+      <c r="E11" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="F11" s="12" t="n">
         <v>0.0081799591002045</v>
       </c>
       <c r="G11" s="5" t="inlineStr">

</xml_diff>